<commit_message>
chore: update coefficients spreadsheet data
</commit_message>
<xml_diff>
--- a/app_unified/public/COEF.xlsx
+++ b/app_unified/public/COEF.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Desktop\ESP DESING ESTUDIO\app_unified\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Desktop\ESP DESING ESTUDIO\ESP DESING ESTUDIO\app_unified\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13EF2173-DF3D-4E0B-9B95-B2ED56E31FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869C1456-8468-45DB-929A-89C69AC578E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FC341EB1-65C7-47F8-9E2D-590F22EBE9EA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">MOTORS!$A$3:$AH$293</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PUMP!$A$2:$AJ$2</definedName>
   </definedNames>
-  <calcPr calcId="191028" concurrentCalc="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -313,7 +313,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1559" uniqueCount="643">
   <si>
     <t>Required Pump data</t>
   </si>
@@ -2289,6 +2289,12 @@
   <si>
     <t>WE-2700</t>
   </si>
+  <si>
+    <t>Baker Hughes</t>
+  </si>
+  <si>
+    <t>P155</t>
+  </si>
 </sst>
 </file>
 
@@ -19202,7 +19208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="14" t="s">
         <v>522</v>
       </c>
@@ -19296,7 +19302,7 @@
       <c r="AE161" s="101"/>
       <c r="AF161" s="98"/>
     </row>
-    <row r="162" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="14" t="s">
         <v>523</v>
       </c>
@@ -19394,7 +19400,117 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="164" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="14" t="s">
+        <v>641</v>
+      </c>
+      <c r="B163" s="93">
+        <v>562</v>
+      </c>
+      <c r="C163" s="93" t="s">
+        <v>642</v>
+      </c>
+      <c r="D163" s="93">
+        <v>11000</v>
+      </c>
+      <c r="E163" s="93">
+        <v>16000</v>
+      </c>
+      <c r="F163" s="93">
+        <v>18500</v>
+      </c>
+      <c r="G163" s="93">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="H163" s="93">
+        <v>24.66</v>
+      </c>
+      <c r="I163" s="93">
+        <v>26000</v>
+      </c>
+      <c r="J163" s="72">
+        <v>60</v>
+      </c>
+      <c r="K163" s="78">
+        <v>24.7</v>
+      </c>
+      <c r="L163" s="78">
+        <v>-7.7700000000000002E-4</v>
+      </c>
+      <c r="M163" s="78">
+        <v>3.8799999999999997E-8</v>
+      </c>
+      <c r="N163" s="78">
+        <v>3.5899999999999998E-12</v>
+      </c>
+      <c r="O163" s="78">
+        <v>-3.9999999999999999E-16</v>
+      </c>
+      <c r="P163" s="78">
+        <v>7.4900000000000001E-21</v>
+      </c>
+      <c r="Q163" s="44">
+        <v>5.16</v>
+      </c>
+      <c r="R163" s="78">
+        <v>-1.44E-4</v>
+      </c>
+      <c r="S163" s="78">
+        <v>4.2499999999999997E-8</v>
+      </c>
+      <c r="T163" s="78">
+        <v>-6.4599999999999997E-13</v>
+      </c>
+      <c r="U163" s="78">
+        <v>-7.3999999999999995E-17</v>
+      </c>
+      <c r="V163" s="78">
+        <v>1.89E-21</v>
+      </c>
+      <c r="W163" s="80">
+        <v>5.62</v>
+      </c>
+      <c r="X163" s="100">
+        <v>5000</v>
+      </c>
+      <c r="Y163" s="100">
+        <v>7500</v>
+      </c>
+      <c r="Z163" s="82">
+        <v>1</v>
+      </c>
+      <c r="AA163" s="100">
+        <v>5.5</v>
+      </c>
+      <c r="AB163" s="100">
+        <v>7.5</v>
+      </c>
+      <c r="AC163" s="101">
+        <v>1</v>
+      </c>
+      <c r="AD163" s="101">
+        <v>45</v>
+      </c>
+      <c r="AE163" s="101">
+        <v>1</v>
+      </c>
+      <c r="AF163" s="98">
+        <v>5200</v>
+      </c>
+      <c r="AG163" s="44" t="s">
+        <v>485</v>
+      </c>
+      <c r="AH163" s="44" t="s">
+        <v>485</v>
+      </c>
+      <c r="AI163" s="44">
+        <v>0</v>
+      </c>
+      <c r="AJ163" s="44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="32"/>
       <c r="B164" s="27"/>
       <c r="C164" s="33"/>
@@ -19428,7 +19544,7 @@
       <c r="AE164" s="31"/>
       <c r="AF164" s="36"/>
     </row>
-    <row r="165" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="32"/>
       <c r="B165" s="27"/>
       <c r="C165" s="33"/>
@@ -19462,7 +19578,7 @@
       <c r="AE165" s="31"/>
       <c r="AF165" s="36"/>
     </row>
-    <row r="166" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="32"/>
       <c r="B166" s="27"/>
       <c r="C166" s="33"/>
@@ -19496,7 +19612,7 @@
       <c r="AE166" s="31"/>
       <c r="AF166" s="36"/>
     </row>
-    <row r="167" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="32"/>
       <c r="B167" s="27"/>
       <c r="C167" s="33"/>
@@ -19530,7 +19646,7 @@
       <c r="AE167" s="31"/>
       <c r="AF167" s="36"/>
     </row>
-    <row r="168" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="32"/>
       <c r="B168" s="27"/>
       <c r="C168" s="33"/>
@@ -19564,7 +19680,7 @@
       <c r="AE168" s="31"/>
       <c r="AF168" s="36"/>
     </row>
-    <row r="169" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="32"/>
       <c r="B169" s="27"/>
       <c r="C169" s="33"/>
@@ -19598,7 +19714,7 @@
       <c r="AE169" s="31"/>
       <c r="AF169" s="36"/>
     </row>
-    <row r="170" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="32"/>
       <c r="B170" s="27"/>
       <c r="C170" s="33"/>
@@ -19634,7 +19750,7 @@
       <c r="AG170" s="45"/>
       <c r="AH170" s="45"/>
     </row>
-    <row r="171" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="32"/>
       <c r="B171" s="27"/>
       <c r="C171" s="33"/>
@@ -19668,7 +19784,7 @@
       <c r="AE171" s="31"/>
       <c r="AF171" s="36"/>
     </row>
-    <row r="172" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="32"/>
       <c r="B172" s="27"/>
       <c r="C172" s="33"/>
@@ -19702,7 +19818,7 @@
       <c r="AE172" s="31"/>
       <c r="AF172" s="36"/>
     </row>
-    <row r="173" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="32"/>
       <c r="B173" s="27"/>
       <c r="C173" s="33"/>
@@ -19736,7 +19852,7 @@
       <c r="AE173" s="31"/>
       <c r="AF173" s="36"/>
     </row>
-    <row r="174" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="32"/>
       <c r="B174" s="27"/>
       <c r="C174" s="33"/>
@@ -19770,7 +19886,7 @@
       <c r="AE174" s="31"/>
       <c r="AF174" s="36"/>
     </row>
-    <row r="175" spans="1:34" s="46" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:36" s="46" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="32"/>
       <c r="B175" s="27"/>
       <c r="C175" s="33"/>
@@ -19804,7 +19920,7 @@
       <c r="AE175" s="31"/>
       <c r="AF175" s="38"/>
     </row>
-    <row r="176" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:36" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="32"/>
       <c r="B176" s="27"/>
       <c r="C176" s="33"/>

</xml_diff>